<commit_message>
update content evidence templates
</commit_message>
<xml_diff>
--- a/back/storage/templates_evidencia/template_evidencia_mmc_epp.xlsx
+++ b/back/storage/templates_evidencia/template_evidencia_mmc_epp.xlsx
@@ -4,15 +4,140 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="MMC-EPP" state="visible" r:id="rId3"/>
+    <sheet sheetId="1" name="Verificación MMC-EPP" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="40">
+  <si>
+    <t>VERIFICACIÓN MANEJO MANUAL DE CARGAS / USO EPP</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Dependencia</t>
+  </si>
+  <si>
+    <t>Inspector</t>
+  </si>
+  <si>
+    <t>SECCIÓN 1: MANEJO MANUAL DE CARGAS (MMC)</t>
+  </si>
+  <si>
+    <t>N°</t>
+  </si>
+  <si>
+    <t>Aspecto a Verificar</t>
+  </si>
+  <si>
+    <t>Cumple</t>
+  </si>
+  <si>
+    <t>No Cumple</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Observación</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Peso de carga ≤ 25 kg (hombres) / 20 kg (mujeres)</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Técnica de levantamiento correcta (piernas, espalda recta)</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Uso de ayudas mecánicas cuando corresponde</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Frecuencia de manipulación dentro de lo permitido</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Almacenamiento de cargas a altura adecuada</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Señalización de pesos en cargas</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Capacitación vigente en MMC</t>
+  </si>
+  <si>
+    <t>SECCIÓN 2: EQUIPOS DE PROTECCIÓN PERSONAL (EPP)</t>
+  </si>
+  <si>
+    <t>Elemento de Protección</t>
+  </si>
+  <si>
+    <t>Casco de seguridad</t>
+  </si>
+  <si>
+    <t>Lentes de seguridad</t>
+  </si>
+  <si>
+    <t>Zapatos de seguridad</t>
+  </si>
+  <si>
+    <t>Guantes de trabajo</t>
+  </si>
+  <si>
+    <t>Ropa de algodón (no sintética)</t>
+  </si>
+  <si>
+    <t>Chaleco reflectante</t>
+  </si>
+  <si>
+    <t>Protección auditiva</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Protección respiratoria</t>
+  </si>
+  <si>
+    <t>Firma Inspector</t>
+  </si>
+  <si>
+    <t>Firma Trabajador</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -20,16 +145,63 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="374151"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="6B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003594"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="475569"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -37,12 +209,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -382,12 +579,441 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:F27"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>